<commit_message>
Improved build scripts Standalone kernel for Forecr boards for L4T >= 36
</commit_message>
<xml_diff>
--- a/MIPI_deployment.xlsx
+++ b/MIPI_deployment.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\CGE\mipi_jetson-l4t-2.0.0\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cyril.germaine\Documents\work\projets\MIPI\mipi_l4t_eg_main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7C152CB-84EF-4D77-BF93-96D5AE6F1FFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE2BA830-4891-4DBD-AFEC-D377BD96B8F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{D61E0E21-A3C2-41B9-A323-5A81E21B33EC}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{D61E0E21-A3C2-41B9-A323-5A81E21B33EC}"/>
   </bookViews>
   <sheets>
     <sheet name="Jetson drivers status" sheetId="5" r:id="rId1"/>
@@ -222,34 +222,12 @@
 Auvidea X230D (tested)</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="5"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Specific build : forecr
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Forecr DSBOARD ORNXS (Orin NX tested)</t>
-    </r>
-  </si>
-  <si>
     <t>Jetson Xavier NX developer kit (tested)
 Waveshare JETSON-IO-BASE-B (tested)
 Seeed A206 carrier board (tested)</t>
+  </si>
+  <si>
+    <t>Forecr DSBOARD ORNXS (tested)</t>
   </si>
 </sst>
 </file>
@@ -259,7 +237,7 @@
   <numFmts count="1">
     <numFmt numFmtId="44" formatCode="_-* #,##0.00\ &quot;€&quot;_-;\-* #,##0.00\ &quot;€&quot;_-;_-* &quot;-&quot;??\ &quot;€&quot;_-;_-@_-"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -279,14 +257,6 @@
       <u/>
       <sz val="11"/>
       <color theme="10"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color theme="5"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -504,7 +474,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="97">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -730,7 +700,53 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -738,20 +754,16 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="8" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -759,43 +771,7 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="5" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="5" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <extLst>
         <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
@@ -803,13 +779,67 @@
         </ext>
       </extLst>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="5" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="8" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -836,83 +866,23 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <extLst>
-        <ext xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
-          <xfpb:xfComplement i="0"/>
-        </ext>
-      </extLst>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1368,8 +1338,8 @@
     <col min="3" max="3" width="13.7109375" customWidth="1"/>
     <col min="4" max="4" width="7.85546875" customWidth="1"/>
     <col min="5" max="5" width="10.85546875" customWidth="1"/>
-    <col min="6" max="6" width="10.42578125" customWidth="1"/>
-    <col min="7" max="7" width="13.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.42578125" style="97" customWidth="1"/>
+    <col min="7" max="7" width="13.85546875" style="97" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="7.7109375" customWidth="1"/>
     <col min="9" max="9" width="11" customWidth="1"/>
     <col min="10" max="10" width="11.85546875" customWidth="1"/>
@@ -1388,202 +1358,202 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="45" x14ac:dyDescent="0.25">
-      <c r="A1" s="44" t="s">
+      <c r="A1" s="43" t="s">
         <v>36</v>
       </c>
-      <c r="B1" s="46" t="s">
+      <c r="B1" s="45" t="s">
         <v>35</v>
       </c>
-      <c r="C1" s="45"/>
+      <c r="C1" s="44"/>
     </row>
     <row r="2" spans="1:21" ht="45" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="B2" s="79" t="s">
+      <c r="B2" s="76" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="79"/>
-      <c r="D2" s="79"/>
-      <c r="E2" s="79"/>
-      <c r="F2" s="83" t="s">
+      <c r="C2" s="76"/>
+      <c r="D2" s="76"/>
+      <c r="E2" s="76"/>
+      <c r="F2" s="80" t="s">
         <v>28</v>
       </c>
-      <c r="G2" s="83"/>
-      <c r="H2" s="83"/>
-      <c r="I2" s="83"/>
-      <c r="J2" s="66" t="s">
-        <v>1</v>
-      </c>
-      <c r="K2" s="66"/>
-      <c r="L2" s="66"/>
-      <c r="M2" s="66"/>
-      <c r="N2" s="70" t="s">
+      <c r="G2" s="80"/>
+      <c r="H2" s="80"/>
+      <c r="I2" s="80"/>
+      <c r="J2" s="86" t="s">
+        <v>1</v>
+      </c>
+      <c r="K2" s="86"/>
+      <c r="L2" s="86"/>
+      <c r="M2" s="86"/>
+      <c r="N2" s="90" t="s">
         <v>34</v>
       </c>
-      <c r="O2" s="70"/>
-      <c r="P2" s="70"/>
-      <c r="Q2" s="70"/>
-      <c r="R2" s="70"/>
-      <c r="S2" s="70"/>
-      <c r="T2" s="70"/>
-      <c r="U2" s="70"/>
+      <c r="O2" s="90"/>
+      <c r="P2" s="90"/>
+      <c r="Q2" s="90"/>
+      <c r="R2" s="90"/>
+      <c r="S2" s="90"/>
+      <c r="T2" s="90"/>
+      <c r="U2" s="90"/>
     </row>
     <row r="3" spans="1:21" ht="46.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
         <v>47</v>
       </c>
-      <c r="B3" s="80" t="s">
+      <c r="B3" s="77" t="s">
         <v>48</v>
       </c>
-      <c r="C3" s="81"/>
-      <c r="D3" s="81"/>
-      <c r="E3" s="82"/>
-      <c r="F3" s="84" t="s">
+      <c r="C3" s="78"/>
+      <c r="D3" s="78"/>
+      <c r="E3" s="79"/>
+      <c r="F3" s="81" t="s">
+        <v>52</v>
+      </c>
+      <c r="G3" s="82"/>
+      <c r="H3" s="82"/>
+      <c r="I3" s="83"/>
+      <c r="J3" s="87" t="s">
+        <v>51</v>
+      </c>
+      <c r="K3" s="88"/>
+      <c r="L3" s="88"/>
+      <c r="M3" s="89"/>
+      <c r="N3" s="91" t="s">
+        <v>49</v>
+      </c>
+      <c r="O3" s="92"/>
+      <c r="P3" s="92"/>
+      <c r="Q3" s="93"/>
+      <c r="R3" s="91" t="s">
         <v>53</v>
       </c>
-      <c r="G3" s="85"/>
-      <c r="H3" s="85"/>
-      <c r="I3" s="86"/>
-      <c r="J3" s="67" t="s">
-        <v>51</v>
-      </c>
-      <c r="K3" s="68"/>
-      <c r="L3" s="68"/>
-      <c r="M3" s="69"/>
-      <c r="N3" s="71" t="s">
-        <v>49</v>
-      </c>
-      <c r="O3" s="72"/>
-      <c r="P3" s="72"/>
-      <c r="Q3" s="73"/>
-      <c r="R3" s="71" t="s">
-        <v>52</v>
-      </c>
-      <c r="S3" s="72"/>
-      <c r="T3" s="72"/>
-      <c r="U3" s="73"/>
+      <c r="S3" s="92"/>
+      <c r="T3" s="92"/>
+      <c r="U3" s="93"/>
     </row>
     <row r="4" spans="1:21" ht="6" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="52"/>
-      <c r="B4" s="54"/>
-      <c r="C4" s="47"/>
-      <c r="D4" s="47"/>
-      <c r="E4" s="55"/>
-      <c r="F4" s="58"/>
-      <c r="G4" s="48"/>
-      <c r="H4" s="48"/>
-      <c r="I4" s="59"/>
-      <c r="J4" s="54"/>
-      <c r="K4" s="47"/>
-      <c r="L4" s="47"/>
-      <c r="M4" s="55"/>
-      <c r="N4" s="54"/>
-      <c r="O4" s="47"/>
-      <c r="P4" s="47"/>
-      <c r="Q4" s="55"/>
-      <c r="R4" s="54"/>
-      <c r="S4" s="47"/>
-      <c r="T4" s="47"/>
-      <c r="U4" s="55"/>
+      <c r="A4" s="49"/>
+      <c r="B4" s="51"/>
+      <c r="C4" s="46"/>
+      <c r="D4" s="46"/>
+      <c r="E4" s="52"/>
+      <c r="F4" s="55"/>
+      <c r="G4" s="47"/>
+      <c r="H4" s="47"/>
+      <c r="I4" s="56"/>
+      <c r="J4" s="51"/>
+      <c r="K4" s="46"/>
+      <c r="L4" s="46"/>
+      <c r="M4" s="52"/>
+      <c r="N4" s="51"/>
+      <c r="O4" s="46"/>
+      <c r="P4" s="46"/>
+      <c r="Q4" s="52"/>
+      <c r="R4" s="51"/>
+      <c r="S4" s="46"/>
+      <c r="T4" s="46"/>
+      <c r="U4" s="52"/>
     </row>
     <row r="5" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="74" t="s">
+      <c r="A5" s="72" t="s">
         <v>50</v>
       </c>
-      <c r="B5" s="92" t="s">
+      <c r="B5" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="75"/>
-      <c r="D5" s="75" t="s">
+      <c r="C5" s="67"/>
+      <c r="D5" s="67" t="s">
         <v>26</v>
       </c>
-      <c r="E5" s="76" t="s">
+      <c r="E5" s="73" t="s">
         <v>27</v>
       </c>
-      <c r="F5" s="77" t="s">
+      <c r="F5" s="74" t="s">
         <v>25</v>
       </c>
-      <c r="G5" s="78"/>
-      <c r="H5" s="87" t="s">
+      <c r="G5" s="75"/>
+      <c r="H5" s="84" t="s">
         <v>26</v>
       </c>
-      <c r="I5" s="88" t="s">
+      <c r="I5" s="85" t="s">
         <v>27</v>
       </c>
-      <c r="J5" s="89" t="s">
+      <c r="J5" s="63" t="s">
         <v>25</v>
       </c>
-      <c r="K5" s="90"/>
-      <c r="L5" s="91" t="s">
+      <c r="K5" s="64"/>
+      <c r="L5" s="65" t="s">
         <v>26</v>
       </c>
-      <c r="M5" s="95" t="s">
+      <c r="M5" s="70" t="s">
         <v>27</v>
       </c>
-      <c r="N5" s="96" t="s">
+      <c r="N5" s="71" t="s">
         <v>25</v>
       </c>
-      <c r="O5" s="93"/>
-      <c r="P5" s="93" t="s">
+      <c r="O5" s="68"/>
+      <c r="P5" s="68" t="s">
         <v>26</v>
       </c>
-      <c r="Q5" s="94" t="s">
+      <c r="Q5" s="69" t="s">
         <v>27</v>
       </c>
-      <c r="R5" s="96" t="s">
+      <c r="R5" s="71" t="s">
         <v>25</v>
       </c>
-      <c r="S5" s="93"/>
-      <c r="T5" s="93" t="s">
+      <c r="S5" s="68"/>
+      <c r="T5" s="68" t="s">
         <v>26</v>
       </c>
-      <c r="U5" s="94" t="s">
+      <c r="U5" s="69" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:21" ht="60" x14ac:dyDescent="0.25">
-      <c r="A6" s="74"/>
+      <c r="A6" s="72"/>
       <c r="B6" s="33" t="s">
         <v>37</v>
       </c>
-      <c r="C6" s="50" t="s">
+      <c r="C6" s="48" t="s">
         <v>38</v>
       </c>
-      <c r="D6" s="75"/>
-      <c r="E6" s="76"/>
+      <c r="D6" s="67"/>
+      <c r="E6" s="73"/>
       <c r="F6" s="40" t="s">
         <v>37</v>
       </c>
-      <c r="G6" s="51" t="s">
+      <c r="G6" s="94" t="s">
         <v>38</v>
       </c>
-      <c r="H6" s="87"/>
-      <c r="I6" s="88"/>
+      <c r="H6" s="84"/>
+      <c r="I6" s="85"/>
       <c r="J6" s="41" t="s">
         <v>37</v>
       </c>
-      <c r="K6" s="49" t="s">
+      <c r="K6" s="95" t="s">
         <v>38</v>
       </c>
-      <c r="L6" s="91"/>
-      <c r="M6" s="95"/>
+      <c r="L6" s="65"/>
+      <c r="M6" s="70"/>
       <c r="N6" s="42" t="s">
         <v>37</v>
       </c>
-      <c r="O6" s="43" t="s">
+      <c r="O6" s="96" t="s">
         <v>38</v>
       </c>
-      <c r="P6" s="93"/>
-      <c r="Q6" s="94"/>
+      <c r="P6" s="68"/>
+      <c r="Q6" s="69"/>
       <c r="R6" s="42" t="s">
         <v>37</v>
       </c>
-      <c r="S6" s="43" t="s">
+      <c r="S6" s="96" t="s">
         <v>38</v>
       </c>
-      <c r="T6" s="93"/>
-      <c r="U6" s="94"/>
+      <c r="T6" s="68"/>
+      <c r="U6" s="69"/>
     </row>
     <row r="7" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="32" t="s">
@@ -1598,7 +1568,7 @@
       <c r="D7" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="E7" s="56" t="s">
+      <c r="E7" s="53" t="s">
         <v>30</v>
       </c>
       <c r="F7" s="28" t="b">
@@ -1663,7 +1633,7 @@
       <c r="D8" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="E8" s="56" t="s">
+      <c r="E8" s="53" t="s">
         <v>30</v>
       </c>
       <c r="F8" s="28" t="b">
@@ -1728,7 +1698,7 @@
       <c r="D9" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="E9" s="56" t="s">
+      <c r="E9" s="53" t="s">
         <v>30</v>
       </c>
       <c r="F9" s="28" t="b">
@@ -1781,7 +1751,7 @@
       </c>
     </row>
     <row r="10" spans="1:21" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="53" t="s">
+      <c r="A10" s="50" t="s">
         <v>2</v>
       </c>
       <c r="B10" s="34" t="b">
@@ -1793,7 +1763,7 @@
       <c r="D10" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="E10" s="57" t="s">
+      <c r="E10" s="54" t="s">
         <v>41</v>
       </c>
       <c r="F10" s="28" t="b">
@@ -1808,10 +1778,10 @@
       <c r="I10" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="J10" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="K10" s="17" t="s">
+      <c r="J10" s="99" t="s">
+        <v>40</v>
+      </c>
+      <c r="K10" s="99" t="s">
         <v>40</v>
       </c>
       <c r="L10" s="17" t="s">
@@ -1820,10 +1790,10 @@
       <c r="M10" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="N10" s="20" t="s">
-        <v>40</v>
-      </c>
-      <c r="O10" s="19" t="s">
+      <c r="N10" s="100" t="s">
+        <v>40</v>
+      </c>
+      <c r="O10" s="100" t="s">
         <v>40</v>
       </c>
       <c r="P10" s="19" t="s">
@@ -1832,10 +1802,10 @@
       <c r="Q10" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="R10" s="20" t="s">
-        <v>40</v>
-      </c>
-      <c r="S10" s="20" t="s">
+      <c r="R10" s="100" t="s">
+        <v>40</v>
+      </c>
+      <c r="S10" s="100" t="s">
         <v>40</v>
       </c>
       <c r="T10" s="19" t="s">
@@ -1846,7 +1816,7 @@
       </c>
     </row>
     <row r="11" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="53" t="s">
+      <c r="A11" s="50" t="s">
         <v>3</v>
       </c>
       <c r="B11" s="34" t="b">
@@ -1858,7 +1828,7 @@
       <c r="D11" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="E11" s="57" t="s">
+      <c r="E11" s="54" t="s">
         <v>41</v>
       </c>
       <c r="F11" s="28" t="b">
@@ -1873,10 +1843,10 @@
       <c r="I11" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="J11" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="K11" s="17" t="s">
+      <c r="J11" s="99" t="s">
+        <v>40</v>
+      </c>
+      <c r="K11" s="99" t="s">
         <v>40</v>
       </c>
       <c r="L11" s="17" t="s">
@@ -1885,10 +1855,10 @@
       <c r="M11" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="N11" s="20" t="s">
-        <v>40</v>
-      </c>
-      <c r="O11" s="19" t="s">
+      <c r="N11" s="100" t="s">
+        <v>40</v>
+      </c>
+      <c r="O11" s="100" t="s">
         <v>40</v>
       </c>
       <c r="P11" s="19" t="s">
@@ -1897,10 +1867,10 @@
       <c r="Q11" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="R11" s="20" t="s">
-        <v>40</v>
-      </c>
-      <c r="S11" s="20" t="s">
+      <c r="R11" s="100" t="s">
+        <v>40</v>
+      </c>
+      <c r="S11" s="100" t="s">
         <v>40</v>
       </c>
       <c r="T11" s="19" t="s">
@@ -1911,7 +1881,7 @@
       </c>
     </row>
     <row r="12" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="53" t="s">
+      <c r="A12" s="50" t="s">
         <v>45</v>
       </c>
       <c r="B12" s="34" t="b">
@@ -1923,7 +1893,7 @@
       <c r="D12" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="E12" s="57" t="s">
+      <c r="E12" s="54" t="s">
         <v>41</v>
       </c>
       <c r="F12" s="28" t="b">
@@ -1938,10 +1908,10 @@
       <c r="I12" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="J12" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="K12" s="17" t="s">
+      <c r="J12" s="99" t="s">
+        <v>40</v>
+      </c>
+      <c r="K12" s="99" t="s">
         <v>40</v>
       </c>
       <c r="L12" s="17" t="s">
@@ -1950,10 +1920,10 @@
       <c r="M12" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="N12" s="20" t="s">
-        <v>40</v>
-      </c>
-      <c r="O12" s="19" t="s">
+      <c r="N12" s="100" t="s">
+        <v>40</v>
+      </c>
+      <c r="O12" s="100" t="s">
         <v>40</v>
       </c>
       <c r="P12" s="19" t="s">
@@ -1962,10 +1932,10 @@
       <c r="Q12" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="R12" s="20" t="s">
-        <v>40</v>
-      </c>
-      <c r="S12" s="20" t="s">
+      <c r="R12" s="100" t="s">
+        <v>40</v>
+      </c>
+      <c r="S12" s="100" t="s">
         <v>40</v>
       </c>
       <c r="T12" s="19" t="s">
@@ -1976,7 +1946,7 @@
       </c>
     </row>
     <row r="13" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="53" t="s">
+      <c r="A13" s="50" t="s">
         <v>46</v>
       </c>
       <c r="B13" s="34" t="b">
@@ -1988,7 +1958,7 @@
       <c r="D13" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="E13" s="57" t="s">
+      <c r="E13" s="54" t="s">
         <v>41</v>
       </c>
       <c r="F13" s="28" t="b">
@@ -2003,10 +1973,10 @@
       <c r="I13" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="J13" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="K13" s="17" t="s">
+      <c r="J13" s="99" t="s">
+        <v>40</v>
+      </c>
+      <c r="K13" s="99" t="s">
         <v>40</v>
       </c>
       <c r="L13" s="17" t="s">
@@ -2015,10 +1985,10 @@
       <c r="M13" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="N13" s="20" t="s">
-        <v>40</v>
-      </c>
-      <c r="O13" s="19" t="s">
+      <c r="N13" s="100" t="s">
+        <v>40</v>
+      </c>
+      <c r="O13" s="100" t="s">
         <v>40</v>
       </c>
       <c r="P13" s="19" t="s">
@@ -2027,10 +1997,10 @@
       <c r="Q13" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="R13" s="20" t="s">
-        <v>40</v>
-      </c>
-      <c r="S13" s="20" t="s">
+      <c r="R13" s="100" t="s">
+        <v>40</v>
+      </c>
+      <c r="S13" s="100" t="s">
         <v>40</v>
       </c>
       <c r="T13" s="19" t="s">
@@ -2041,7 +2011,7 @@
       </c>
     </row>
     <row r="14" spans="1:21" ht="36" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="53" t="s">
+      <c r="A14" s="50" t="s">
         <v>4</v>
       </c>
       <c r="B14" s="35" t="s">
@@ -2065,7 +2035,7 @@
       <c r="H14" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="I14" s="60" t="s">
+      <c r="I14" s="57" t="s">
         <v>41</v>
       </c>
       <c r="J14" s="24" t="b">
@@ -2080,10 +2050,10 @@
       <c r="M14" s="25" t="s">
         <v>29</v>
       </c>
-      <c r="N14" s="20" t="s">
-        <v>40</v>
-      </c>
-      <c r="O14" s="19" t="s">
+      <c r="N14" s="100" t="s">
+        <v>40</v>
+      </c>
+      <c r="O14" s="100" t="s">
         <v>40</v>
       </c>
       <c r="P14" s="19" t="s">
@@ -2092,10 +2062,10 @@
       <c r="Q14" s="21" t="s">
         <v>29</v>
       </c>
-      <c r="R14" s="20" t="s">
-        <v>40</v>
-      </c>
-      <c r="S14" s="20" t="s">
+      <c r="R14" s="100" t="s">
+        <v>40</v>
+      </c>
+      <c r="S14" s="100" t="s">
         <v>40</v>
       </c>
       <c r="T14" s="19" t="s">
@@ -2106,7 +2076,7 @@
       </c>
     </row>
     <row r="15" spans="1:21" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="53" t="s">
+      <c r="A15" s="50" t="s">
         <v>5</v>
       </c>
       <c r="B15" s="35" t="s">
@@ -2130,7 +2100,7 @@
       <c r="H15" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="I15" s="60" t="s">
+      <c r="I15" s="57" t="s">
         <v>41</v>
       </c>
       <c r="J15" s="24" t="b">
@@ -2142,7 +2112,7 @@
       <c r="L15" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="M15" s="61" t="s">
+      <c r="M15" s="58" t="s">
         <v>41</v>
       </c>
       <c r="N15" s="20" t="b">
@@ -2151,17 +2121,17 @@
       <c r="O15" s="19" t="b">
         <v>1</v>
       </c>
-      <c r="P15" s="65" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q15" s="62" t="s">
+      <c r="P15" s="62" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q15" s="59" t="s">
         <v>41</v>
       </c>
       <c r="R15" s="20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S15" s="19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T15" s="19" t="s">
         <v>29</v>
@@ -2171,7 +2141,7 @@
       </c>
     </row>
     <row r="16" spans="1:21" ht="36.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="53" t="s">
+      <c r="A16" s="50" t="s">
         <v>6</v>
       </c>
       <c r="B16" s="35" t="s">
@@ -2195,7 +2165,7 @@
       <c r="H16" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="I16" s="60" t="s">
+      <c r="I16" s="57" t="s">
         <v>41</v>
       </c>
       <c r="J16" s="24" t="b">
@@ -2207,7 +2177,7 @@
       <c r="L16" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="M16" s="61" t="s">
+      <c r="M16" s="58" t="s">
         <v>41</v>
       </c>
       <c r="N16" s="20" t="b">
@@ -2216,17 +2186,17 @@
       <c r="O16" s="19" t="b">
         <v>1</v>
       </c>
-      <c r="P16" s="65" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q16" s="62" t="s">
+      <c r="P16" s="62" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q16" s="59" t="s">
         <v>41</v>
       </c>
       <c r="R16" s="20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S16" s="19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T16" s="19" t="s">
         <v>29</v>
@@ -2236,7 +2206,7 @@
       </c>
     </row>
     <row r="17" spans="1:21" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="53" t="s">
+      <c r="A17" s="50" t="s">
         <v>7</v>
       </c>
       <c r="B17" s="35" t="s">
@@ -2260,7 +2230,7 @@
       <c r="H17" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="I17" s="60" t="s">
+      <c r="I17" s="57" t="s">
         <v>41</v>
       </c>
       <c r="J17" s="24" t="b">
@@ -2272,7 +2242,7 @@
       <c r="L17" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="M17" s="61" t="s">
+      <c r="M17" s="58" t="s">
         <v>41</v>
       </c>
       <c r="N17" s="20" t="b">
@@ -2281,17 +2251,17 @@
       <c r="O17" s="19" t="b">
         <v>1</v>
       </c>
-      <c r="P17" s="65" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q17" s="62" t="s">
+      <c r="P17" s="62" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q17" s="59" t="s">
         <v>41</v>
       </c>
       <c r="R17" s="20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S17" s="19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T17" s="19" t="s">
         <v>29</v>
@@ -2301,7 +2271,7 @@
       </c>
     </row>
     <row r="18" spans="1:21" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="53" t="s">
+      <c r="A18" s="50" t="s">
         <v>42</v>
       </c>
       <c r="B18" s="35" t="s">
@@ -2325,7 +2295,7 @@
       <c r="H18" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="I18" s="60" t="s">
+      <c r="I18" s="57" t="s">
         <v>41</v>
       </c>
       <c r="J18" s="24" t="b">
@@ -2337,7 +2307,7 @@
       <c r="L18" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="M18" s="61" t="s">
+      <c r="M18" s="58" t="s">
         <v>41</v>
       </c>
       <c r="N18" s="20" t="b">
@@ -2346,17 +2316,17 @@
       <c r="O18" s="19" t="b">
         <v>1</v>
       </c>
-      <c r="P18" s="65" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q18" s="62" t="s">
+      <c r="P18" s="62" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q18" s="59" t="s">
         <v>41</v>
       </c>
       <c r="R18" s="20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S18" s="19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T18" s="19" t="s">
         <v>29</v>
@@ -2366,7 +2336,7 @@
       </c>
     </row>
     <row r="19" spans="1:21" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="53" t="s">
+      <c r="A19" s="50" t="s">
         <v>43</v>
       </c>
       <c r="B19" s="35" t="s">
@@ -2390,7 +2360,7 @@
       <c r="H19" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="I19" s="60" t="s">
+      <c r="I19" s="57" t="s">
         <v>41</v>
       </c>
       <c r="J19" s="24" t="b">
@@ -2402,7 +2372,7 @@
       <c r="L19" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="M19" s="61" t="s">
+      <c r="M19" s="58" t="s">
         <v>41</v>
       </c>
       <c r="N19" s="20" t="b">
@@ -2411,17 +2381,17 @@
       <c r="O19" s="19" t="b">
         <v>1</v>
       </c>
-      <c r="P19" s="65" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q19" s="62" t="s">
+      <c r="P19" s="62" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q19" s="59" t="s">
         <v>41</v>
       </c>
       <c r="R19" s="20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S19" s="19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T19" s="19" t="s">
         <v>29</v>
@@ -2431,7 +2401,7 @@
       </c>
     </row>
     <row r="20" spans="1:21" ht="33.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="53" t="s">
+      <c r="A20" s="50" t="s">
         <v>44</v>
       </c>
       <c r="B20" s="35" t="s">
@@ -2455,7 +2425,7 @@
       <c r="H20" s="16" t="s">
         <v>33</v>
       </c>
-      <c r="I20" s="60" t="s">
+      <c r="I20" s="57" t="s">
         <v>41</v>
       </c>
       <c r="J20" s="24" t="b">
@@ -2467,7 +2437,7 @@
       <c r="L20" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="M20" s="61" t="s">
+      <c r="M20" s="58" t="s">
         <v>41</v>
       </c>
       <c r="N20" s="20" t="b">
@@ -2476,17 +2446,17 @@
       <c r="O20" s="19" t="b">
         <v>1</v>
       </c>
-      <c r="P20" s="65" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q20" s="62" t="s">
+      <c r="P20" s="62" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q20" s="59" t="s">
         <v>41</v>
       </c>
       <c r="R20" s="20" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S20" s="19" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T20" s="19" t="s">
         <v>29</v>
@@ -2496,7 +2466,7 @@
       </c>
     </row>
     <row r="21" spans="1:21" ht="45" x14ac:dyDescent="0.25">
-      <c r="A21" s="53" t="s">
+      <c r="A21" s="50" t="s">
         <v>31</v>
       </c>
       <c r="B21" s="35" t="s">
@@ -2511,10 +2481,10 @@
       <c r="E21" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="F21" s="28" t="s">
-        <v>40</v>
-      </c>
-      <c r="G21" s="28" t="s">
+      <c r="F21" s="98" t="s">
+        <v>40</v>
+      </c>
+      <c r="G21" s="98" t="s">
         <v>40</v>
       </c>
       <c r="H21" s="15" t="s">
@@ -2532,7 +2502,7 @@
       <c r="L21" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="M21" s="61" t="s">
+      <c r="M21" s="58" t="s">
         <v>41</v>
       </c>
       <c r="N21" s="20" t="b">
@@ -2541,10 +2511,10 @@
       <c r="O21" s="19" t="b">
         <v>1</v>
       </c>
-      <c r="P21" s="65" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q21" s="62" t="s">
+      <c r="P21" s="62" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q21" s="59" t="s">
         <v>41</v>
       </c>
       <c r="R21" s="20" t="b">
@@ -2553,15 +2523,15 @@
       <c r="S21" s="19" t="b">
         <v>1</v>
       </c>
-      <c r="T21" s="65" t="s">
-        <v>33</v>
-      </c>
-      <c r="U21" s="62" t="s">
+      <c r="T21" s="62" t="s">
+        <v>33</v>
+      </c>
+      <c r="U21" s="59" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="22" spans="1:21" ht="45" x14ac:dyDescent="0.25">
-      <c r="A22" s="53" t="s">
+      <c r="A22" s="50" t="s">
         <v>24</v>
       </c>
       <c r="B22" s="35" t="s">
@@ -2576,10 +2546,10 @@
       <c r="E22" s="36" t="s">
         <v>29</v>
       </c>
-      <c r="F22" s="28" t="s">
-        <v>40</v>
-      </c>
-      <c r="G22" s="28" t="s">
+      <c r="F22" s="98" t="s">
+        <v>40</v>
+      </c>
+      <c r="G22" s="98" t="s">
         <v>40</v>
       </c>
       <c r="H22" s="15" t="s">
@@ -2597,7 +2567,7 @@
       <c r="L22" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="M22" s="61" t="s">
+      <c r="M22" s="58" t="s">
         <v>41</v>
       </c>
       <c r="N22" s="20" t="b">
@@ -2606,10 +2576,10 @@
       <c r="O22" s="19" t="b">
         <v>1</v>
       </c>
-      <c r="P22" s="65" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q22" s="63" t="s">
+      <c r="P22" s="62" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q22" s="60" t="s">
         <v>41</v>
       </c>
       <c r="R22" s="20" t="b">
@@ -2618,15 +2588,15 @@
       <c r="S22" s="19" t="b">
         <v>1</v>
       </c>
-      <c r="T22" s="65" t="s">
-        <v>33</v>
-      </c>
-      <c r="U22" s="63" t="s">
+      <c r="T22" s="62" t="s">
+        <v>33</v>
+      </c>
+      <c r="U22" s="60" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="23" spans="1:21" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A23" s="53" t="s">
+      <c r="A23" s="50" t="s">
         <v>32</v>
       </c>
       <c r="B23" s="37" t="s">
@@ -2641,10 +2611,10 @@
       <c r="E23" s="39" t="s">
         <v>29</v>
       </c>
-      <c r="F23" s="28" t="s">
-        <v>40</v>
-      </c>
-      <c r="G23" s="28" t="s">
+      <c r="F23" s="98" t="s">
+        <v>40</v>
+      </c>
+      <c r="G23" s="98" t="s">
         <v>40</v>
       </c>
       <c r="H23" s="30" t="s">
@@ -2662,7 +2632,7 @@
       <c r="L23" s="18" t="s">
         <v>33</v>
       </c>
-      <c r="M23" s="61" t="s">
+      <c r="M23" s="58" t="s">
         <v>41</v>
       </c>
       <c r="N23" s="22" t="b">
@@ -2671,10 +2641,10 @@
       <c r="O23" s="23" t="b">
         <v>1</v>
       </c>
-      <c r="P23" s="65" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q23" s="64" t="s">
+      <c r="P23" s="62" t="s">
+        <v>33</v>
+      </c>
+      <c r="Q23" s="61" t="s">
         <v>41</v>
       </c>
       <c r="R23" s="22" t="b">
@@ -2683,16 +2653,31 @@
       <c r="S23" s="23" t="b">
         <v>1</v>
       </c>
-      <c r="T23" s="65" t="s">
-        <v>33</v>
-      </c>
-      <c r="U23" s="64" t="s">
+      <c r="T23" s="62" t="s">
+        <v>33</v>
+      </c>
+      <c r="U23" s="61" t="s">
         <v>41</v>
       </c>
     </row>
     <row r="24" spans="1:21" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="J2:M2"/>
+    <mergeCell ref="J3:M3"/>
+    <mergeCell ref="N2:U2"/>
+    <mergeCell ref="N3:Q3"/>
+    <mergeCell ref="R3:U3"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F2:I2"/>
+    <mergeCell ref="F3:I3"/>
+    <mergeCell ref="H5:H6"/>
+    <mergeCell ref="I5:I6"/>
     <mergeCell ref="J5:K5"/>
     <mergeCell ref="L5:L6"/>
     <mergeCell ref="B5:C5"/>
@@ -2703,21 +2688,6 @@
     <mergeCell ref="P5:P6"/>
     <mergeCell ref="Q5:Q6"/>
     <mergeCell ref="R5:S5"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F2:I2"/>
-    <mergeCell ref="F3:I3"/>
-    <mergeCell ref="H5:H6"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="J2:M2"/>
-    <mergeCell ref="J3:M3"/>
-    <mergeCell ref="N2:U2"/>
-    <mergeCell ref="N3:Q3"/>
-    <mergeCell ref="R3:U3"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="D7" r:id="rId1" xr:uid="{E221AAD3-4BB4-4EDE-B796-266DB5695C55}"/>
@@ -2887,6 +2857,33 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="ddfcbff1-988c-4780-af66-42272a7444f2" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5eab2033-26a9-4886-8f5a-efa3f46bf7e3">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <SharedWithUsers xmlns="ddfcbff1-988c-4780-af66-42272a7444f2">
+      <UserInfo>
+        <DisplayName>Cyril Germaine</DisplayName>
+        <AccountId>370</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100994F61C2E354C24B867AAD14EB9B712B" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="173ead120da22e4d04d58d9334952390">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="5eab2033-26a9-4886-8f5a-efa3f46bf7e3" xmlns:ns3="ddfcbff1-988c-4780-af66-42272a7444f2" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="7ed80a0b9a34c83decd038c2f8c861fc" ns2:_="" ns3:_="">
     <xsd:import namespace="5eab2033-26a9-4886-8f5a-efa3f46bf7e3"/>
@@ -3141,34 +3138,32 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C6CC26F4-9ACA-496B-B719-4372C9693134}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="5eab2033-26a9-4886-8f5a-efa3f46bf7e3"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="ddfcbff1-988c-4780-af66-42272a7444f2"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="ddfcbff1-988c-4780-af66-42272a7444f2" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="5eab2033-26a9-4886-8f5a-efa3f46bf7e3">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <SharedWithUsers xmlns="ddfcbff1-988c-4780-af66-42272a7444f2">
-      <UserInfo>
-        <DisplayName>Cyril Germaine</DisplayName>
-        <AccountId>370</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{21273CB7-CC8A-48C1-BA2A-0CD67C70C578}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{31B71CDC-0E86-4889-96FE-F63C9CD1A6C7}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -3185,29 +3180,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{21273CB7-CC8A-48C1-BA2A-0CD67C70C578}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C6CC26F4-9ACA-496B-B719-4372C9693134}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="5eab2033-26a9-4886-8f5a-efa3f46bf7e3"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="ddfcbff1-988c-4780-af66-42272a7444f2"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
Removed AGX Orin L4T 36.4.4
</commit_message>
<xml_diff>
--- a/MIPI_deployment.xlsx
+++ b/MIPI_deployment.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\CGE\mipi_jetson-l4t-2.0.0\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cyril.germaine\Documents\work\projets\MIPI\mipi_l4t_eg_main\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7C152CB-84EF-4D77-BF93-96D5AE6F1FFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C94CFB7C-64C6-4540-9D4C-E4C15A500229}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="25440" windowHeight="15270" xr2:uid="{D61E0E21-A3C2-41B9-A323-5A81E21B33EC}"/>
   </bookViews>
@@ -812,75 +812,6 @@
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <extLst>
@@ -903,6 +834,9 @@
     <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -913,6 +847,72 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="9" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1412,22 +1412,22 @@
       <c r="G2" s="83"/>
       <c r="H2" s="83"/>
       <c r="I2" s="83"/>
-      <c r="J2" s="66" t="s">
-        <v>1</v>
-      </c>
-      <c r="K2" s="66"/>
-      <c r="L2" s="66"/>
-      <c r="M2" s="66"/>
-      <c r="N2" s="70" t="s">
+      <c r="J2" s="89" t="s">
+        <v>1</v>
+      </c>
+      <c r="K2" s="89"/>
+      <c r="L2" s="89"/>
+      <c r="M2" s="89"/>
+      <c r="N2" s="93" t="s">
         <v>34</v>
       </c>
-      <c r="O2" s="70"/>
-      <c r="P2" s="70"/>
-      <c r="Q2" s="70"/>
-      <c r="R2" s="70"/>
-      <c r="S2" s="70"/>
-      <c r="T2" s="70"/>
-      <c r="U2" s="70"/>
+      <c r="O2" s="93"/>
+      <c r="P2" s="93"/>
+      <c r="Q2" s="93"/>
+      <c r="R2" s="93"/>
+      <c r="S2" s="93"/>
+      <c r="T2" s="93"/>
+      <c r="U2" s="93"/>
     </row>
     <row r="3" spans="1:21" ht="46.5" customHeight="1" thickTop="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
@@ -1445,24 +1445,24 @@
       <c r="G3" s="85"/>
       <c r="H3" s="85"/>
       <c r="I3" s="86"/>
-      <c r="J3" s="67" t="s">
+      <c r="J3" s="90" t="s">
         <v>51</v>
       </c>
-      <c r="K3" s="68"/>
-      <c r="L3" s="68"/>
-      <c r="M3" s="69"/>
-      <c r="N3" s="71" t="s">
+      <c r="K3" s="91"/>
+      <c r="L3" s="91"/>
+      <c r="M3" s="92"/>
+      <c r="N3" s="94" t="s">
         <v>49</v>
       </c>
-      <c r="O3" s="72"/>
-      <c r="P3" s="72"/>
-      <c r="Q3" s="73"/>
-      <c r="R3" s="71" t="s">
+      <c r="O3" s="95"/>
+      <c r="P3" s="95"/>
+      <c r="Q3" s="96"/>
+      <c r="R3" s="94" t="s">
         <v>52</v>
       </c>
-      <c r="S3" s="72"/>
-      <c r="T3" s="72"/>
-      <c r="U3" s="73"/>
+      <c r="S3" s="95"/>
+      <c r="T3" s="95"/>
+      <c r="U3" s="96"/>
     </row>
     <row r="4" spans="1:21" ht="6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="52"/>
@@ -1488,14 +1488,14 @@
       <c r="U4" s="55"/>
     </row>
     <row r="5" spans="1:21" ht="29.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="74" t="s">
+      <c r="A5" s="75" t="s">
         <v>50</v>
       </c>
-      <c r="B5" s="92" t="s">
+      <c r="B5" s="69" t="s">
         <v>25</v>
       </c>
-      <c r="C5" s="75"/>
-      <c r="D5" s="75" t="s">
+      <c r="C5" s="70"/>
+      <c r="D5" s="70" t="s">
         <v>26</v>
       </c>
       <c r="E5" s="76" t="s">
@@ -1511,46 +1511,46 @@
       <c r="I5" s="88" t="s">
         <v>27</v>
       </c>
-      <c r="J5" s="89" t="s">
+      <c r="J5" s="66" t="s">
         <v>25</v>
       </c>
-      <c r="K5" s="90"/>
-      <c r="L5" s="91" t="s">
+      <c r="K5" s="67"/>
+      <c r="L5" s="68" t="s">
         <v>26</v>
       </c>
-      <c r="M5" s="95" t="s">
+      <c r="M5" s="73" t="s">
         <v>27</v>
       </c>
-      <c r="N5" s="96" t="s">
+      <c r="N5" s="74" t="s">
         <v>25</v>
       </c>
-      <c r="O5" s="93"/>
-      <c r="P5" s="93" t="s">
+      <c r="O5" s="71"/>
+      <c r="P5" s="71" t="s">
         <v>26</v>
       </c>
-      <c r="Q5" s="94" t="s">
+      <c r="Q5" s="72" t="s">
         <v>27</v>
       </c>
-      <c r="R5" s="96" t="s">
+      <c r="R5" s="74" t="s">
         <v>25</v>
       </c>
-      <c r="S5" s="93"/>
-      <c r="T5" s="93" t="s">
+      <c r="S5" s="71"/>
+      <c r="T5" s="71" t="s">
         <v>26</v>
       </c>
-      <c r="U5" s="94" t="s">
+      <c r="U5" s="72" t="s">
         <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:21" ht="60" x14ac:dyDescent="0.25">
-      <c r="A6" s="74"/>
+      <c r="A6" s="75"/>
       <c r="B6" s="33" t="s">
         <v>37</v>
       </c>
       <c r="C6" s="50" t="s">
         <v>38</v>
       </c>
-      <c r="D6" s="75"/>
+      <c r="D6" s="70"/>
       <c r="E6" s="76"/>
       <c r="F6" s="40" t="s">
         <v>37</v>
@@ -1566,24 +1566,24 @@
       <c r="K6" s="49" t="s">
         <v>38</v>
       </c>
-      <c r="L6" s="91"/>
-      <c r="M6" s="95"/>
+      <c r="L6" s="68"/>
+      <c r="M6" s="73"/>
       <c r="N6" s="42" t="s">
         <v>37</v>
       </c>
       <c r="O6" s="43" t="s">
         <v>38</v>
       </c>
-      <c r="P6" s="93"/>
-      <c r="Q6" s="94"/>
+      <c r="P6" s="71"/>
+      <c r="Q6" s="72"/>
       <c r="R6" s="42" t="s">
         <v>37</v>
       </c>
       <c r="S6" s="43" t="s">
         <v>38</v>
       </c>
-      <c r="T6" s="93"/>
-      <c r="U6" s="94"/>
+      <c r="T6" s="71"/>
+      <c r="U6" s="72"/>
     </row>
     <row r="7" spans="1:21" ht="30" hidden="1" x14ac:dyDescent="0.25">
       <c r="A7" s="32" t="s">
@@ -2560,7 +2560,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="22" spans="1:21" ht="45" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:21" ht="30" x14ac:dyDescent="0.25">
       <c r="A22" s="53" t="s">
         <v>24</v>
       </c>
@@ -2625,7 +2625,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="23" spans="1:21" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:21" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="53" t="s">
         <v>32</v>
       </c>
@@ -2654,16 +2654,16 @@
         <v>29</v>
       </c>
       <c r="J23" s="26" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="K23" s="27" t="b">
-        <v>1</v>
-      </c>
-      <c r="L23" s="18" t="s">
-        <v>33</v>
-      </c>
-      <c r="M23" s="61" t="s">
-        <v>41</v>
+        <v>0</v>
+      </c>
+      <c r="L23" s="27" t="s">
+        <v>29</v>
+      </c>
+      <c r="M23" s="27" t="s">
+        <v>29</v>
       </c>
       <c r="N23" s="22" t="b">
         <v>1</v>
@@ -2693,6 +2693,21 @@
     <row r="24" spans="1:21" ht="15.75" thickTop="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="J2:M2"/>
+    <mergeCell ref="J3:M3"/>
+    <mergeCell ref="N2:U2"/>
+    <mergeCell ref="N3:Q3"/>
+    <mergeCell ref="R3:U3"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="F5:G5"/>
+    <mergeCell ref="B2:E2"/>
+    <mergeCell ref="B3:E3"/>
+    <mergeCell ref="F2:I2"/>
+    <mergeCell ref="F3:I3"/>
+    <mergeCell ref="H5:H6"/>
+    <mergeCell ref="I5:I6"/>
     <mergeCell ref="J5:K5"/>
     <mergeCell ref="L5:L6"/>
     <mergeCell ref="B5:C5"/>
@@ -2703,21 +2718,6 @@
     <mergeCell ref="P5:P6"/>
     <mergeCell ref="Q5:Q6"/>
     <mergeCell ref="R5:S5"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="F5:G5"/>
-    <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="F2:I2"/>
-    <mergeCell ref="F3:I3"/>
-    <mergeCell ref="H5:H6"/>
-    <mergeCell ref="I5:I6"/>
-    <mergeCell ref="J2:M2"/>
-    <mergeCell ref="J3:M3"/>
-    <mergeCell ref="N2:U2"/>
-    <mergeCell ref="N3:Q3"/>
-    <mergeCell ref="R3:U3"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="D7" r:id="rId1" xr:uid="{E221AAD3-4BB4-4EDE-B796-266DB5695C55}"/>
@@ -2767,27 +2767,25 @@
     <hyperlink ref="E13" r:id="rId45" xr:uid="{5479132F-A40A-48BD-B01F-26EC045D6E2A}"/>
     <hyperlink ref="L21" r:id="rId46" xr:uid="{42D2EEFE-31E1-4354-AB23-366FC1B50B3B}"/>
     <hyperlink ref="L22" r:id="rId47" xr:uid="{6145CAE4-C0F2-47E0-8D13-BC66CB770D29}"/>
-    <hyperlink ref="L23" r:id="rId48" xr:uid="{D47B40AC-FACA-49B1-B20B-D09A03BA8AD9}"/>
-    <hyperlink ref="Q15" r:id="rId49" xr:uid="{B47F3C8B-316E-443E-9A83-924E035001F5}"/>
-    <hyperlink ref="P15" r:id="rId50" xr:uid="{45826816-8105-43D7-877C-49D91AB45DFF}"/>
-    <hyperlink ref="Q16" r:id="rId51" xr:uid="{99C02D54-E95B-406E-888C-11B77A415407}"/>
-    <hyperlink ref="P16" r:id="rId52" xr:uid="{FD01E274-56E3-4F2F-A2BD-6648C48F8601}"/>
-    <hyperlink ref="Q17" r:id="rId53" xr:uid="{3AC0B3F2-CE34-43E1-B289-37A16A325A80}"/>
-    <hyperlink ref="P17" r:id="rId54" xr:uid="{80B0D63D-BE27-4F41-A640-4AA6D933C698}"/>
-    <hyperlink ref="Q18" r:id="rId55" xr:uid="{0186A2C2-BD40-4092-A5ED-EECA3BA42D33}"/>
-    <hyperlink ref="P18" r:id="rId56" xr:uid="{A0AB0304-5ED5-4C36-9090-DEA65BBC836D}"/>
-    <hyperlink ref="Q19" r:id="rId57" xr:uid="{56F2E20D-76E2-4691-A147-D5FE7F94FA6B}"/>
-    <hyperlink ref="P19" r:id="rId58" xr:uid="{555AFD0B-AEE7-4AA4-9D7E-F1BAA3BF173C}"/>
-    <hyperlink ref="Q20" r:id="rId59" xr:uid="{43EB682D-C577-4144-9CA9-005673003CE8}"/>
-    <hyperlink ref="P20" r:id="rId60" xr:uid="{D71B2251-121D-458C-A2E2-DEC71E37F921}"/>
-    <hyperlink ref="M16" r:id="rId61" xr:uid="{223B3D30-B82E-4315-AF84-8D55398EC1E6}"/>
-    <hyperlink ref="M17" r:id="rId62" xr:uid="{9A33580F-2891-41A7-8471-13DDC5C0606E}"/>
-    <hyperlink ref="M18" r:id="rId63" xr:uid="{B7F95591-3680-4FD6-987A-A8BB624D85BB}"/>
-    <hyperlink ref="M19" r:id="rId64" xr:uid="{2A59B455-3361-40C9-AB82-4D0D8413D619}"/>
-    <hyperlink ref="M20" r:id="rId65" xr:uid="{761859F5-06A9-41B3-B623-2548209B824E}"/>
-    <hyperlink ref="M21" r:id="rId66" xr:uid="{C31471EA-AE7D-4471-BC33-F9AF319B883B}"/>
-    <hyperlink ref="M22" r:id="rId67" xr:uid="{97359225-836C-4AE2-BBFA-336A691A912D}"/>
-    <hyperlink ref="M23" r:id="rId68" xr:uid="{E102F9C9-438D-4172-AFDA-EC2CD812DF66}"/>
+    <hyperlink ref="Q15" r:id="rId48" xr:uid="{B47F3C8B-316E-443E-9A83-924E035001F5}"/>
+    <hyperlink ref="P15" r:id="rId49" xr:uid="{45826816-8105-43D7-877C-49D91AB45DFF}"/>
+    <hyperlink ref="Q16" r:id="rId50" xr:uid="{99C02D54-E95B-406E-888C-11B77A415407}"/>
+    <hyperlink ref="P16" r:id="rId51" xr:uid="{FD01E274-56E3-4F2F-A2BD-6648C48F8601}"/>
+    <hyperlink ref="Q17" r:id="rId52" xr:uid="{3AC0B3F2-CE34-43E1-B289-37A16A325A80}"/>
+    <hyperlink ref="P17" r:id="rId53" xr:uid="{80B0D63D-BE27-4F41-A640-4AA6D933C698}"/>
+    <hyperlink ref="Q18" r:id="rId54" xr:uid="{0186A2C2-BD40-4092-A5ED-EECA3BA42D33}"/>
+    <hyperlink ref="P18" r:id="rId55" xr:uid="{A0AB0304-5ED5-4C36-9090-DEA65BBC836D}"/>
+    <hyperlink ref="Q19" r:id="rId56" xr:uid="{56F2E20D-76E2-4691-A147-D5FE7F94FA6B}"/>
+    <hyperlink ref="P19" r:id="rId57" xr:uid="{555AFD0B-AEE7-4AA4-9D7E-F1BAA3BF173C}"/>
+    <hyperlink ref="Q20" r:id="rId58" xr:uid="{43EB682D-C577-4144-9CA9-005673003CE8}"/>
+    <hyperlink ref="P20" r:id="rId59" xr:uid="{D71B2251-121D-458C-A2E2-DEC71E37F921}"/>
+    <hyperlink ref="M16" r:id="rId60" xr:uid="{223B3D30-B82E-4315-AF84-8D55398EC1E6}"/>
+    <hyperlink ref="M17" r:id="rId61" xr:uid="{9A33580F-2891-41A7-8471-13DDC5C0606E}"/>
+    <hyperlink ref="M18" r:id="rId62" xr:uid="{B7F95591-3680-4FD6-987A-A8BB624D85BB}"/>
+    <hyperlink ref="M19" r:id="rId63" xr:uid="{2A59B455-3361-40C9-AB82-4D0D8413D619}"/>
+    <hyperlink ref="M20" r:id="rId64" xr:uid="{761859F5-06A9-41B3-B623-2548209B824E}"/>
+    <hyperlink ref="M21" r:id="rId65" xr:uid="{C31471EA-AE7D-4471-BC33-F9AF319B883B}"/>
+    <hyperlink ref="M22" r:id="rId66" xr:uid="{97359225-836C-4AE2-BBFA-336A691A912D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3142,15 +3140,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="ddfcbff1-988c-4780-af66-42272a7444f2" xsi:nil="true"/>
@@ -3166,6 +3155,15 @@
     </SharedWithUsers>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3188,14 +3186,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{21273CB7-CC8A-48C1-BA2A-0CD67C70C578}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C6CC26F4-9ACA-496B-B719-4372C9693134}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="5eab2033-26a9-4886-8f5a-efa3f46bf7e3"/>
@@ -3210,4 +3200,12 @@
     <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{21273CB7-CC8A-48C1-BA2A-0CD67C70C578}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>